<commit_message>
Plein de petites modifications
</commit_message>
<xml_diff>
--- a/Debut/utils/correspondance_echo_final.xlsx
+++ b/Debut/utils/correspondance_echo_final.xlsx
@@ -45088,7 +45088,9 @@
       <c r="N802" t="n">
         <v>191</v>
       </c>
-      <c r="O802" t="inlineStr"/>
+      <c r="O802" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="803">
       <c r="A803" t="n">
@@ -45143,7 +45145,9 @@
       <c r="N803" t="n">
         <v>191</v>
       </c>
-      <c r="O803" t="inlineStr"/>
+      <c r="O803" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="804">
       <c r="A804" t="n">
@@ -45198,7 +45202,9 @@
       <c r="N804" t="n">
         <v>191</v>
       </c>
-      <c r="O804" t="inlineStr"/>
+      <c r="O804" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="805">
       <c r="A805" t="n">
@@ -45845,7 +45851,7 @@
         <v>191</v>
       </c>
       <c r="O816" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="817">
@@ -45902,7 +45908,7 @@
         <v>191</v>
       </c>
       <c r="O817" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="818">
@@ -45959,7 +45965,7 @@
         <v>191</v>
       </c>
       <c r="O818" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="819">
@@ -46004,7 +46010,7 @@
         <v>191</v>
       </c>
       <c r="O819" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="820">
@@ -51803,7 +51809,7 @@
         <v>288</v>
       </c>
       <c r="O924" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="925">
@@ -51864,7 +51870,7 @@
         <v>288</v>
       </c>
       <c r="O925" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="926">
@@ -51925,7 +51931,7 @@
         <v>288</v>
       </c>
       <c r="O926" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="927">
@@ -51986,7 +51992,7 @@
         <v>288</v>
       </c>
       <c r="O927" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="928">
@@ -52047,7 +52053,7 @@
         <v>288</v>
       </c>
       <c r="O928" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="929">
@@ -52096,7 +52102,7 @@
         <v>288</v>
       </c>
       <c r="O929" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="930">

</xml_diff>